<commit_message>
Update mapping audit sheet to add Target Dashboard Tab/Page column
</commit_message>
<xml_diff>
--- a/STEAMEE_Reports_Mapping_Audit.xlsx
+++ b/STEAMEE_Reports_Mapping_Audit.xlsx
@@ -528,7 +528,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I114"/>
+  <dimension ref="A1:J114"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -540,6 +540,7 @@
     <col width="42" customWidth="1" min="7" max="7"/>
     <col width="45" customWidth="1" min="8" max="8"/>
     <col width="45" customWidth="1" min="9" max="9"/>
+    <col width="32" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -595,6 +596,11 @@
           <t>Gaps &amp; Action Items (Dev Work)</t>
         </is>
       </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>Target Dashboard Tab / Page</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="42" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
@@ -642,6 +648,11 @@
           <t>None. Handled by existing data schema.</t>
         </is>
       </c>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>1. Overview Hub, 2. User Analytics, 3. Store Operations, 5. Finance &amp; Revenue, 11. Operational Lists &amp; Tables</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="42" customHeight="1">
       <c r="A4" s="6" t="inlineStr">
@@ -689,6 +700,11 @@
           <t>None. Handled by existing data schema.</t>
         </is>
       </c>
+      <c r="J4" s="6" t="inlineStr">
+        <is>
+          <t>1. Overview Hub, 2. User Analytics, 3. Store Operations, 5. Finance &amp; Revenue, 11. Operational Lists &amp; Tables</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="42" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
@@ -736,6 +752,11 @@
           <t>None. Handled by existing data schema.</t>
         </is>
       </c>
+      <c r="J5" s="3" t="inlineStr">
+        <is>
+          <t>1. Overview Hub, 2. User Analytics, 3. Store Operations, 5. Finance &amp; Revenue, 11. Operational Lists &amp; Tables</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="42" customHeight="1">
       <c r="A6" s="6" t="inlineStr">
@@ -783,6 +804,11 @@
           <t>None. Handled by existing data schema.</t>
         </is>
       </c>
+      <c r="J6" s="6" t="inlineStr">
+        <is>
+          <t>1. Overview Hub, 2. User Analytics, 3. Store Operations, 5. Finance &amp; Revenue, 11. Operational Lists &amp; Tables</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="42" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
@@ -830,6 +856,11 @@
           <t>None. Handled by existing data schema.</t>
         </is>
       </c>
+      <c r="J7" s="3" t="inlineStr">
+        <is>
+          <t>1. Overview Hub, 2. User Analytics, 3. Store Operations, 5. Finance &amp; Revenue, 11. Operational Lists &amp; Tables</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="42" customHeight="1">
       <c r="A8" s="6" t="inlineStr">
@@ -877,6 +908,11 @@
           <t>None. Handled by existing data schema.</t>
         </is>
       </c>
+      <c r="J8" s="6" t="inlineStr">
+        <is>
+          <t>1. Overview Hub, 2. User Analytics, 3. Store Operations, 5. Finance &amp; Revenue, 11. Operational Lists &amp; Tables</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="42" customHeight="1">
       <c r="A9" s="3" t="inlineStr">
@@ -924,6 +960,11 @@
           <t>None. Handled by existing data schema.</t>
         </is>
       </c>
+      <c r="J9" s="3" t="inlineStr">
+        <is>
+          <t>2. User Analytics</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="42" customHeight="1">
       <c r="A10" s="6" t="inlineStr">
@@ -971,6 +1012,11 @@
           <t>None. Handled by existing data schema.</t>
         </is>
       </c>
+      <c r="J10" s="6" t="inlineStr">
+        <is>
+          <t>2. User Analytics</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="42" customHeight="1">
       <c r="A11" s="3" t="inlineStr">
@@ -1018,6 +1064,11 @@
           <t>None. Handled by existing data schema.</t>
         </is>
       </c>
+      <c r="J11" s="3" t="inlineStr">
+        <is>
+          <t>1. Overview Hub, 2. User Analytics, 3. Store Operations, 7. Complaint &amp; Quality</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="42" customHeight="1">
       <c r="A12" s="6" t="inlineStr">
@@ -1065,6 +1116,11 @@
           <t>None. Handled by existing data schema.</t>
         </is>
       </c>
+      <c r="J12" s="6" t="inlineStr">
+        <is>
+          <t>1. Overview Hub, 2. User Analytics, 3. Store Operations, 7. Complaint &amp; Quality</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="42" customHeight="1">
       <c r="A13" s="3" t="inlineStr">
@@ -1112,6 +1168,11 @@
           <t>None.</t>
         </is>
       </c>
+      <c r="J13" s="3" t="inlineStr">
+        <is>
+          <t>1. Overview Hub, 2. User Analytics, 3. Store Operations, 7. Complaint &amp; Quality</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="42" customHeight="1">
       <c r="A14" s="6" t="inlineStr">
@@ -1159,6 +1220,11 @@
           <t>None. Handled by existing data schema.</t>
         </is>
       </c>
+      <c r="J14" s="6" t="inlineStr">
+        <is>
+          <t>1. Overview Hub, 2. User Analytics, 5. Finance &amp; Revenue, 11. Operational Lists &amp; Tables</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="42" customHeight="1">
       <c r="A15" s="3" t="inlineStr">
@@ -1206,6 +1272,11 @@
           <t>None. Handled by existing data schema.</t>
         </is>
       </c>
+      <c r="J15" s="3" t="inlineStr">
+        <is>
+          <t>1. Overview Hub, 2. User Analytics, 5. Finance &amp; Revenue, 11. Operational Lists &amp; Tables</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="42" customHeight="1">
       <c r="A16" s="6" t="inlineStr">
@@ -1253,6 +1324,11 @@
           <t>None. Handled by existing data schema.</t>
         </is>
       </c>
+      <c r="J16" s="6" t="inlineStr">
+        <is>
+          <t>6. Growth &amp; Marketing</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="42" customHeight="1">
       <c r="A17" s="3" t="inlineStr">
@@ -1300,6 +1376,11 @@
           <t>None. Handled by existing data schema.</t>
         </is>
       </c>
+      <c r="J17" s="3" t="inlineStr">
+        <is>
+          <t>5. Finance &amp; Revenue</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="42" customHeight="1">
       <c r="A18" s="6" t="inlineStr">
@@ -1347,6 +1428,11 @@
           <t>None. Handled by existing data schema.</t>
         </is>
       </c>
+      <c r="J18" s="6" t="inlineStr">
+        <is>
+          <t>5. Finance &amp; Revenue</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="42" customHeight="1">
       <c r="A19" s="3" t="inlineStr">
@@ -1394,6 +1480,11 @@
           <t>None. Handled by existing data schema.</t>
         </is>
       </c>
+      <c r="J19" s="3" t="inlineStr">
+        <is>
+          <t>1. Overview Hub, 2. User Analytics, 5. Finance &amp; Revenue, 11. Operational Lists &amp; Tables</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="42" customHeight="1">
       <c r="A20" s="6" t="inlineStr">
@@ -1441,6 +1532,11 @@
           <t>None. Handled by existing data schema.</t>
         </is>
       </c>
+      <c r="J20" s="6" t="inlineStr">
+        <is>
+          <t>1. Overview Hub, 2. User Analytics, 5. Finance &amp; Revenue</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="42" customHeight="1">
       <c r="A21" s="3" t="inlineStr">
@@ -1488,6 +1584,11 @@
           <t>None. Handled by existing data schema.</t>
         </is>
       </c>
+      <c r="J21" s="3" t="inlineStr">
+        <is>
+          <t>1. Overview Hub, 2. User Analytics, 5. Finance &amp; Revenue, 11. Operational Lists &amp; Tables</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="42" customHeight="1">
       <c r="A22" s="6" t="inlineStr">
@@ -1535,6 +1636,11 @@
           <t>Needs dedicated field for return logistics fee in DB.</t>
         </is>
       </c>
+      <c r="J22" s="6" t="inlineStr">
+        <is>
+          <t>3. Store Operations, 4. Rider Logistics, 5. Finance &amp; Revenue, 8. TAT Analytics</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="42" customHeight="1">
       <c r="A23" s="3" t="inlineStr">
@@ -1582,6 +1688,11 @@
           <t>None.</t>
         </is>
       </c>
+      <c r="J23" s="3" t="inlineStr">
+        <is>
+          <t>2. User Analytics, 5. Finance &amp; Revenue, 7. Complaint &amp; Quality</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="42" customHeight="1">
       <c r="A24" s="6" t="inlineStr">
@@ -1629,6 +1740,11 @@
           <t>None.</t>
         </is>
       </c>
+      <c r="J24" s="6" t="inlineStr">
+        <is>
+          <t>2. User Analytics, 5. Finance &amp; Revenue, 7. Complaint &amp; Quality</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="42" customHeight="1">
       <c r="A25" s="3" t="inlineStr">
@@ -1676,6 +1792,11 @@
           <t>None.</t>
         </is>
       </c>
+      <c r="J25" s="3" t="inlineStr">
+        <is>
+          <t>2. User Analytics, 5. Finance &amp; Revenue, 7. Complaint &amp; Quality</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="42" customHeight="1">
       <c r="A26" s="6" t="inlineStr">
@@ -1723,6 +1844,11 @@
           <t>None.</t>
         </is>
       </c>
+      <c r="J26" s="6" t="inlineStr">
+        <is>
+          <t>2. User Analytics, 5. Finance &amp; Revenue, 7. Complaint &amp; Quality</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="42" customHeight="1">
       <c r="A27" s="3" t="inlineStr">
@@ -1770,6 +1896,11 @@
           <t>Requires a Metabase timestamp duration logic, not a default card yet.</t>
         </is>
       </c>
+      <c r="J27" s="3" t="inlineStr">
+        <is>
+          <t>2. User Analytics, 5. Finance &amp; Revenue, 7. Complaint &amp; Quality</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="42" customHeight="1">
       <c r="A28" s="6" t="inlineStr">
@@ -1817,6 +1948,11 @@
           <t>None.</t>
         </is>
       </c>
+      <c r="J28" s="6" t="inlineStr">
+        <is>
+          <t>2. User Analytics, 5. Finance &amp; Revenue, 7. Complaint &amp; Quality</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="42" customHeight="1">
       <c r="A29" s="3" t="inlineStr">
@@ -1864,6 +2000,11 @@
           <t>Missing daily opening stock, closing stock, and receipts database logs.</t>
         </is>
       </c>
+      <c r="J29" s="3" t="inlineStr">
+        <is>
+          <t>3. Store Operations</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="42" customHeight="1">
       <c r="A30" s="6" t="inlineStr">
@@ -1911,6 +2052,11 @@
           <t>Missing daily opening stock, closing stock, and receipts database logs.</t>
         </is>
       </c>
+      <c r="J30" s="6" t="inlineStr">
+        <is>
+          <t>3. Store Operations</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="42" customHeight="1">
       <c r="A31" s="3" t="inlineStr">
@@ -1958,6 +2104,11 @@
           <t>Missing daily opening stock, closing stock, and receipts database logs.</t>
         </is>
       </c>
+      <c r="J31" s="3" t="inlineStr">
+        <is>
+          <t>3. Store Operations</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="42" customHeight="1">
       <c r="A32" s="6" t="inlineStr">
@@ -2005,6 +2156,11 @@
           <t>Missing daily opening stock, closing stock, and receipts database logs.</t>
         </is>
       </c>
+      <c r="J32" s="6" t="inlineStr">
+        <is>
+          <t>3. Store Operations</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="42" customHeight="1">
       <c r="A33" s="3" t="inlineStr">
@@ -2052,6 +2208,11 @@
           <t>None. Handled by existing data schema.</t>
         </is>
       </c>
+      <c r="J33" s="3" t="inlineStr">
+        <is>
+          <t>1. Overview Hub, 4. Rider Logistics, 8. TAT Analytics, 11. Operational Lists &amp; Tables</t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="42" customHeight="1">
       <c r="A34" s="6" t="inlineStr">
@@ -2099,6 +2260,11 @@
           <t>None. Handled by existing data schema.</t>
         </is>
       </c>
+      <c r="J34" s="6" t="inlineStr">
+        <is>
+          <t>1. Overview Hub, 8. TAT Analytics, 11. Operational Lists &amp; Tables</t>
+        </is>
+      </c>
     </row>
     <row r="35" ht="42" customHeight="1">
       <c r="A35" s="3" t="inlineStr">
@@ -2146,6 +2312,11 @@
           <t>None. Handled by existing data schema.</t>
         </is>
       </c>
+      <c r="J35" s="3" t="inlineStr">
+        <is>
+          <t>1. Overview Hub, 4. Rider Logistics, 8. TAT Analytics, 11. Operational Lists &amp; Tables</t>
+        </is>
+      </c>
     </row>
     <row r="36" ht="42" customHeight="1">
       <c r="A36" s="6" t="inlineStr">
@@ -2193,6 +2364,11 @@
           <t>None. Handled by existing data schema.</t>
         </is>
       </c>
+      <c r="J36" s="6" t="inlineStr">
+        <is>
+          <t>1. Overview Hub, 8. TAT Analytics, 11. Operational Lists &amp; Tables</t>
+        </is>
+      </c>
     </row>
     <row r="37" ht="42" customHeight="1">
       <c r="A37" s="3" t="inlineStr">
@@ -2240,6 +2416,11 @@
           <t>Missing machine service cost tracking, store maintenance costs, and cleanliness score.</t>
         </is>
       </c>
+      <c r="J37" s="3" t="inlineStr">
+        <is>
+          <t>3. Store Operations</t>
+        </is>
+      </c>
     </row>
     <row r="38" ht="42" customHeight="1">
       <c r="A38" s="6" t="inlineStr">
@@ -2287,6 +2468,11 @@
           <t>Missing machine service cost tracking, store maintenance costs, and cleanliness score.</t>
         </is>
       </c>
+      <c r="J38" s="6" t="inlineStr">
+        <is>
+          <t>3. Store Operations</t>
+        </is>
+      </c>
     </row>
     <row r="39" ht="42" customHeight="1">
       <c r="A39" s="3" t="inlineStr">
@@ -2334,6 +2520,11 @@
           <t>Missing machine service cost tracking, store maintenance costs, and cleanliness score.</t>
         </is>
       </c>
+      <c r="J39" s="3" t="inlineStr">
+        <is>
+          <t>3. Store Operations</t>
+        </is>
+      </c>
     </row>
     <row r="40" ht="42" customHeight="1">
       <c r="A40" s="6" t="inlineStr">
@@ -2381,6 +2572,11 @@
           <t>Missing machine service cost tracking, store maintenance costs, and cleanliness score.</t>
         </is>
       </c>
+      <c r="J40" s="6" t="inlineStr">
+        <is>
+          <t>3. Store Operations</t>
+        </is>
+      </c>
     </row>
     <row r="41" ht="42" customHeight="1">
       <c r="A41" s="3" t="inlineStr">
@@ -2428,6 +2624,11 @@
           <t>Missing pressman KYC status columns.</t>
         </is>
       </c>
+      <c r="J41" s="3" t="inlineStr">
+        <is>
+          <t>9. Ironer &amp; Staff Performance</t>
+        </is>
+      </c>
     </row>
     <row r="42" ht="42" customHeight="1">
       <c r="A42" s="6" t="inlineStr">
@@ -2475,6 +2676,11 @@
           <t>None. Handled by existing data schema.</t>
         </is>
       </c>
+      <c r="J42" s="6" t="inlineStr">
+        <is>
+          <t>1. Overview Hub, 3. Store Operations, 7. Complaint &amp; Quality, 8. TAT Analytics, 9. Ironer &amp; Staff Performance</t>
+        </is>
+      </c>
     </row>
     <row r="43" ht="42" customHeight="1">
       <c r="A43" s="3" t="inlineStr">
@@ -2522,6 +2728,11 @@
           <t>Payout report structure needs formatting on database side (G4).</t>
         </is>
       </c>
+      <c r="J43" s="3" t="inlineStr">
+        <is>
+          <t>1. Overview Hub, 3. Store Operations, 7. Complaint &amp; Quality, 8. TAT Analytics, 9. Ironer &amp; Staff Performance</t>
+        </is>
+      </c>
     </row>
     <row r="44" ht="42" customHeight="1">
       <c r="A44" s="6" t="inlineStr">
@@ -2569,6 +2780,11 @@
           <t>None.</t>
         </is>
       </c>
+      <c r="J44" s="6" t="inlineStr">
+        <is>
+          <t>2. User Analytics, 5. Finance &amp; Revenue, 7. Complaint &amp; Quality</t>
+        </is>
+      </c>
     </row>
     <row r="45" ht="42" customHeight="1">
       <c r="A45" s="3" t="inlineStr">
@@ -2616,6 +2832,11 @@
           <t>Needs barcode scans at every micro-stage in the workshop.</t>
         </is>
       </c>
+      <c r="J45" s="3" t="inlineStr">
+        <is>
+          <t>9. Ironer &amp; Staff Performance</t>
+        </is>
+      </c>
     </row>
     <row r="46" ht="42" customHeight="1">
       <c r="A46" s="6" t="inlineStr">
@@ -2663,6 +2884,11 @@
           <t>Needs barcode scans at every micro-stage in the workshop.</t>
         </is>
       </c>
+      <c r="J46" s="6" t="inlineStr">
+        <is>
+          <t>9. Ironer &amp; Staff Performance</t>
+        </is>
+      </c>
     </row>
     <row r="47" ht="42" customHeight="1">
       <c r="A47" s="3" t="inlineStr">
@@ -2710,6 +2936,11 @@
           <t>Needs barcode scans at every micro-stage in the workshop.</t>
         </is>
       </c>
+      <c r="J47" s="3" t="inlineStr">
+        <is>
+          <t>9. Ironer &amp; Staff Performance</t>
+        </is>
+      </c>
     </row>
     <row r="48" ht="42" customHeight="1">
       <c r="A48" s="6" t="inlineStr">
@@ -2757,6 +2988,11 @@
           <t>None. Handled by existing data schema.</t>
         </is>
       </c>
+      <c r="J48" s="6" t="inlineStr">
+        <is>
+          <t>1. Overview Hub, 3. Store Operations, 7. Complaint &amp; Quality, 8. TAT Analytics, 9. Ironer &amp; Staff Performance</t>
+        </is>
+      </c>
     </row>
     <row r="49" ht="42" customHeight="1">
       <c r="A49" s="3" t="inlineStr">
@@ -2804,6 +3040,11 @@
           <t>No digital marketing spend tracking exists. Blocked by missing marketing spend table.</t>
         </is>
       </c>
+      <c r="J49" s="3" t="inlineStr">
+        <is>
+          <t>6. Growth &amp; Marketing</t>
+        </is>
+      </c>
     </row>
     <row r="50" ht="42" customHeight="1">
       <c r="A50" s="6" t="inlineStr">
@@ -2851,6 +3092,11 @@
           <t>No digital marketing spend tracking exists. Blocked by missing marketing spend table.</t>
         </is>
       </c>
+      <c r="J50" s="6" t="inlineStr">
+        <is>
+          <t>6. Growth &amp; Marketing</t>
+        </is>
+      </c>
     </row>
     <row r="51" ht="42" customHeight="1">
       <c r="A51" s="3" t="inlineStr">
@@ -2898,6 +3144,11 @@
           <t>No digital marketing spend tracking exists. Blocked by missing marketing spend table.</t>
         </is>
       </c>
+      <c r="J51" s="3" t="inlineStr">
+        <is>
+          <t>6. Growth &amp; Marketing</t>
+        </is>
+      </c>
     </row>
     <row r="52" ht="42" customHeight="1">
       <c r="A52" s="6" t="inlineStr">
@@ -2945,6 +3196,11 @@
           <t>No digital marketing spend tracking exists. Blocked by missing marketing spend table.</t>
         </is>
       </c>
+      <c r="J52" s="6" t="inlineStr">
+        <is>
+          <t>6. Growth &amp; Marketing</t>
+        </is>
+      </c>
     </row>
     <row r="53" ht="42" customHeight="1">
       <c r="A53" s="3" t="inlineStr">
@@ -2992,6 +3248,11 @@
           <t>None. Handled by existing data schema.</t>
         </is>
       </c>
+      <c r="J53" s="3" t="inlineStr">
+        <is>
+          <t>1. Overview Hub, 2. User Analytics, 3. Store Operations, 5. Finance &amp; Revenue, 11. Operational Lists &amp; Tables</t>
+        </is>
+      </c>
     </row>
     <row r="54" ht="42" customHeight="1">
       <c r="A54" s="6" t="inlineStr">
@@ -3039,6 +3300,11 @@
           <t>None. Handled by existing data schema.</t>
         </is>
       </c>
+      <c r="J54" s="6" t="inlineStr">
+        <is>
+          <t>1. Overview Hub, 2. User Analytics, 3. Store Operations, 5. Finance &amp; Revenue, 11. Operational Lists &amp; Tables</t>
+        </is>
+      </c>
     </row>
     <row r="55" ht="42" customHeight="1">
       <c r="A55" s="3" t="inlineStr">
@@ -3086,6 +3352,11 @@
           <t>None. Handled by existing data schema.</t>
         </is>
       </c>
+      <c r="J55" s="3" t="inlineStr">
+        <is>
+          <t>1. Overview Hub, 2. User Analytics, 3. Store Operations, 5. Finance &amp; Revenue, 11. Operational Lists &amp; Tables</t>
+        </is>
+      </c>
     </row>
     <row r="56" ht="42" customHeight="1">
       <c r="A56" s="6" t="inlineStr">
@@ -3133,6 +3404,11 @@
           <t>None. Handled by existing data schema.</t>
         </is>
       </c>
+      <c r="J56" s="6" t="inlineStr">
+        <is>
+          <t>1. Overview Hub, 8. TAT Analytics, 11. Operational Lists &amp; Tables</t>
+        </is>
+      </c>
     </row>
     <row r="57" ht="42" customHeight="1">
       <c r="A57" s="3" t="inlineStr">
@@ -3180,6 +3456,11 @@
           <t>None. Handled by existing data schema.</t>
         </is>
       </c>
+      <c r="J57" s="3" t="inlineStr">
+        <is>
+          <t>1. Overview Hub, 8. TAT Analytics, 11. Operational Lists &amp; Tables</t>
+        </is>
+      </c>
     </row>
     <row r="58" ht="42" customHeight="1">
       <c r="A58" s="6" t="inlineStr">
@@ -3227,6 +3508,11 @@
           <t>None. Handled by existing data schema.</t>
         </is>
       </c>
+      <c r="J58" s="6" t="inlineStr">
+        <is>
+          <t>1. Overview Hub, 2. User Analytics, 3. Store Operations, 5. Finance &amp; Revenue, 11. Operational Lists &amp; Tables</t>
+        </is>
+      </c>
     </row>
     <row r="59" ht="42" customHeight="1">
       <c r="A59" s="3" t="inlineStr">
@@ -3274,6 +3560,11 @@
           <t>None. Handled by existing data schema.</t>
         </is>
       </c>
+      <c r="J59" s="3" t="inlineStr">
+        <is>
+          <t>1. Overview Hub, 2. User Analytics, 3. Store Operations, 5. Finance &amp; Revenue, 11. Operational Lists &amp; Tables</t>
+        </is>
+      </c>
     </row>
     <row r="60" ht="42" customHeight="1">
       <c r="A60" s="6" t="inlineStr">
@@ -3321,6 +3612,11 @@
           <t>None. Handled by existing data schema.</t>
         </is>
       </c>
+      <c r="J60" s="6" t="inlineStr">
+        <is>
+          <t>1. Overview Hub, 3. Store Operations, 7. Complaint &amp; Quality, 8. TAT Analytics, 9. Ironer &amp; Staff Performance</t>
+        </is>
+      </c>
     </row>
     <row r="61" ht="42" customHeight="1">
       <c r="A61" s="3" t="inlineStr">
@@ -3368,6 +3664,11 @@
           <t>None. Handled by existing data schema.</t>
         </is>
       </c>
+      <c r="J61" s="3" t="inlineStr">
+        <is>
+          <t>1. Overview Hub, 3. Store Operations, 7. Complaint &amp; Quality, 8. TAT Analytics, 9. Ironer &amp; Staff Performance</t>
+        </is>
+      </c>
     </row>
     <row r="62" ht="42" customHeight="1">
       <c r="A62" s="6" t="inlineStr">
@@ -3415,6 +3716,11 @@
           <t>None. Handled by existing data schema.</t>
         </is>
       </c>
+      <c r="J62" s="6" t="inlineStr">
+        <is>
+          <t>1. Overview Hub, 8. TAT Analytics, 11. Operational Lists &amp; Tables</t>
+        </is>
+      </c>
     </row>
     <row r="63" ht="42" customHeight="1">
       <c r="A63" s="3" t="inlineStr">
@@ -3462,6 +3768,11 @@
           <t>None. Handled by existing data schema.</t>
         </is>
       </c>
+      <c r="J63" s="3" t="inlineStr">
+        <is>
+          <t>1. Overview Hub, 2. User Analytics, 3. Store Operations, 7. Complaint &amp; Quality</t>
+        </is>
+      </c>
     </row>
     <row r="64" ht="42" customHeight="1">
       <c r="A64" s="6" t="inlineStr">
@@ -3509,6 +3820,11 @@
           <t>None. Handled by existing data schema.</t>
         </is>
       </c>
+      <c r="J64" s="6" t="inlineStr">
+        <is>
+          <t>1. Overview Hub, 2. User Analytics, 5. Finance &amp; Revenue, 11. Operational Lists &amp; Tables</t>
+        </is>
+      </c>
     </row>
     <row r="65" ht="42" customHeight="1">
       <c r="A65" s="3" t="inlineStr">
@@ -3556,6 +3872,11 @@
           <t>None. Handled by existing data schema.</t>
         </is>
       </c>
+      <c r="J65" s="3" t="inlineStr">
+        <is>
+          <t>1. Overview Hub, 2. User Analytics, 3. Store Operations, 5. Finance &amp; Revenue, 11. Operational Lists &amp; Tables</t>
+        </is>
+      </c>
     </row>
     <row r="66" ht="42" customHeight="1">
       <c r="A66" s="6" t="inlineStr">
@@ -3603,6 +3924,11 @@
           <t>None. Handled by existing data schema.</t>
         </is>
       </c>
+      <c r="J66" s="6" t="inlineStr">
+        <is>
+          <t>1. Overview Hub, 2. User Analytics, 3. Store Operations, 5. Finance &amp; Revenue, 11. Operational Lists &amp; Tables</t>
+        </is>
+      </c>
     </row>
     <row r="67" ht="42" customHeight="1">
       <c r="A67" s="3" t="inlineStr">
@@ -3650,6 +3976,11 @@
           <t>None.</t>
         </is>
       </c>
+      <c r="J67" s="3" t="inlineStr">
+        <is>
+          <t>2. User Analytics, 5. Finance &amp; Revenue, 7. Complaint &amp; Quality</t>
+        </is>
+      </c>
     </row>
     <row r="68" ht="42" customHeight="1">
       <c r="A68" s="6" t="inlineStr">
@@ -3697,6 +4028,11 @@
           <t>Requires store manager real-time flag for bags delayed beyond 24 hours.</t>
         </is>
       </c>
+      <c r="J68" s="6" t="inlineStr">
+        <is>
+          <t>3. Store Operations</t>
+        </is>
+      </c>
     </row>
     <row r="69" ht="42" customHeight="1">
       <c r="A69" s="3" t="inlineStr">
@@ -3744,6 +4080,11 @@
           <t>None. Handled by existing data schema.</t>
         </is>
       </c>
+      <c r="J69" s="3" t="inlineStr">
+        <is>
+          <t>1. Overview Hub, 2. User Analytics, 3. Store Operations, 5. Finance &amp; Revenue, 11. Operational Lists &amp; Tables</t>
+        </is>
+      </c>
     </row>
     <row r="70" ht="42" customHeight="1">
       <c r="A70" s="6" t="inlineStr">
@@ -3791,6 +4132,11 @@
           <t>None. Handled by existing data schema.</t>
         </is>
       </c>
+      <c r="J70" s="6" t="inlineStr">
+        <is>
+          <t>5. Finance &amp; Revenue</t>
+        </is>
+      </c>
     </row>
     <row r="71" ht="42" customHeight="1">
       <c r="A71" s="3" t="inlineStr">
@@ -3838,6 +4184,11 @@
           <t>None. Handled by existing data schema.</t>
         </is>
       </c>
+      <c r="J71" s="3" t="inlineStr">
+        <is>
+          <t>1. Overview Hub, 2. User Analytics, 3. Store Operations, 5. Finance &amp; Revenue, 11. Operational Lists &amp; Tables</t>
+        </is>
+      </c>
     </row>
     <row r="72" ht="42" customHeight="1">
       <c r="A72" s="6" t="inlineStr">
@@ -3885,6 +4236,11 @@
           <t>None. Handled by existing data schema.</t>
         </is>
       </c>
+      <c r="J72" s="6" t="inlineStr">
+        <is>
+          <t>1. Overview Hub, 2. User Analytics, 3. Store Operations, 5. Finance &amp; Revenue, 11. Operational Lists &amp; Tables</t>
+        </is>
+      </c>
     </row>
     <row r="73" ht="42" customHeight="1">
       <c r="A73" s="3" t="inlineStr">
@@ -3932,6 +4288,11 @@
           <t>None. Handled by existing data schema.</t>
         </is>
       </c>
+      <c r="J73" s="3" t="inlineStr">
+        <is>
+          <t>1. Overview Hub, 2. User Analytics, 3. Store Operations, 7. Complaint &amp; Quality</t>
+        </is>
+      </c>
     </row>
     <row r="74" ht="42" customHeight="1">
       <c r="A74" s="6" t="inlineStr">
@@ -3979,6 +4340,11 @@
           <t>None. Handled by existing data schema.</t>
         </is>
       </c>
+      <c r="J74" s="6" t="inlineStr">
+        <is>
+          <t>5. Finance &amp; Revenue</t>
+        </is>
+      </c>
     </row>
     <row r="75" ht="42" customHeight="1">
       <c r="A75" s="3" t="inlineStr">
@@ -4026,6 +4392,11 @@
           <t>None. Handled by existing data schema.</t>
         </is>
       </c>
+      <c r="J75" s="3" t="inlineStr">
+        <is>
+          <t>1. Overview Hub, 3. Store Operations, 7. Complaint &amp; Quality, 8. TAT Analytics, 9. Ironer &amp; Staff Performance</t>
+        </is>
+      </c>
     </row>
     <row r="76" ht="42" customHeight="1">
       <c r="A76" s="6" t="inlineStr">
@@ -4073,6 +4444,11 @@
           <t>None. Handled by existing data schema.</t>
         </is>
       </c>
+      <c r="J76" s="6" t="inlineStr">
+        <is>
+          <t>1. Overview Hub, 2. User Analytics, 6. Growth &amp; Marketing</t>
+        </is>
+      </c>
     </row>
     <row r="77" ht="42" customHeight="1">
       <c r="A77" s="3" t="inlineStr">
@@ -4120,6 +4496,11 @@
           <t>None. Handled by existing data schema.</t>
         </is>
       </c>
+      <c r="J77" s="3" t="inlineStr">
+        <is>
+          <t>5. Finance &amp; Revenue</t>
+        </is>
+      </c>
     </row>
     <row r="78" ht="42" customHeight="1">
       <c r="A78" s="6" t="inlineStr">
@@ -4167,6 +4548,11 @@
           <t>None. Handled by existing data schema.</t>
         </is>
       </c>
+      <c r="J78" s="6" t="inlineStr">
+        <is>
+          <t>1. Overview Hub, 2. User Analytics, 3. Store Operations, 5. Finance &amp; Revenue, 11. Operational Lists &amp; Tables</t>
+        </is>
+      </c>
     </row>
     <row r="79" ht="42" customHeight="1">
       <c r="A79" s="3" t="inlineStr">
@@ -4214,6 +4600,11 @@
           <t>None. Handled by existing data schema.</t>
         </is>
       </c>
+      <c r="J79" s="3" t="inlineStr">
+        <is>
+          <t>1. Overview Hub, 2. User Analytics, 3. Store Operations, 5. Finance &amp; Revenue, 11. Operational Lists &amp; Tables</t>
+        </is>
+      </c>
     </row>
     <row r="80" ht="42" customHeight="1">
       <c r="A80" s="6" t="inlineStr">
@@ -4261,6 +4652,11 @@
           <t>None. Handled by existing data schema.</t>
         </is>
       </c>
+      <c r="J80" s="6" t="inlineStr">
+        <is>
+          <t>1. Overview Hub, 2. User Analytics, 5. Finance &amp; Revenue, 11. Operational Lists &amp; Tables</t>
+        </is>
+      </c>
     </row>
     <row r="81" ht="42" customHeight="1">
       <c r="A81" s="3" t="inlineStr">
@@ -4308,6 +4704,11 @@
           <t>None. Handled by existing data schema.</t>
         </is>
       </c>
+      <c r="J81" s="3" t="inlineStr">
+        <is>
+          <t>1. Overview Hub, 3. Store Operations, 7. Complaint &amp; Quality, 8. TAT Analytics, 9. Ironer &amp; Staff Performance</t>
+        </is>
+      </c>
     </row>
     <row r="82" ht="42" customHeight="1">
       <c r="A82" s="6" t="inlineStr">
@@ -4355,6 +4756,11 @@
           <t>None.</t>
         </is>
       </c>
+      <c r="J82" s="6" t="inlineStr">
+        <is>
+          <t>1. Overview Hub, 2. User Analytics, 3. Store Operations, 7. Complaint &amp; Quality</t>
+        </is>
+      </c>
     </row>
     <row r="83" ht="42" customHeight="1">
       <c r="A83" s="3" t="inlineStr">
@@ -4402,6 +4808,11 @@
           <t>None. Handled by existing data schema.</t>
         </is>
       </c>
+      <c r="J83" s="3" t="inlineStr">
+        <is>
+          <t>1. Overview Hub, 2. User Analytics, 3. Store Operations, 5. Finance &amp; Revenue, 11. Operational Lists &amp; Tables</t>
+        </is>
+      </c>
     </row>
     <row r="84" ht="42" customHeight="1">
       <c r="A84" s="6" t="inlineStr">
@@ -4449,6 +4860,11 @@
           <t>None. Handled by existing data schema.</t>
         </is>
       </c>
+      <c r="J84" s="6" t="inlineStr">
+        <is>
+          <t>3. Store Operations, 11. Operational Lists &amp; Tables</t>
+        </is>
+      </c>
     </row>
     <row r="85" ht="42" customHeight="1">
       <c r="A85" s="3" t="inlineStr">
@@ -4496,6 +4912,11 @@
           <t>Requires integration with MoEngage or Clevertap for event-driven message triggers.</t>
         </is>
       </c>
+      <c r="J85" s="3" t="inlineStr">
+        <is>
+          <t>7. Complaint &amp; Quality (RTO) &amp; MoEngage</t>
+        </is>
+      </c>
     </row>
     <row r="86" ht="42" customHeight="1">
       <c r="A86" s="6" t="inlineStr">
@@ -4543,6 +4964,11 @@
           <t>None.</t>
         </is>
       </c>
+      <c r="J86" s="6" t="inlineStr">
+        <is>
+          <t>10. Masters Configuration</t>
+        </is>
+      </c>
     </row>
     <row r="87" ht="42" customHeight="1">
       <c r="A87" s="3" t="inlineStr">
@@ -4590,6 +5016,11 @@
           <t>Need pincode field mapped in orders and users APIs to track sales, cohorts, and slot trends.</t>
         </is>
       </c>
+      <c r="J87" s="3" t="inlineStr">
+        <is>
+          <t>3. Store Operations &amp; 2. User Analytics</t>
+        </is>
+      </c>
     </row>
     <row r="88" ht="42" customHeight="1">
       <c r="A88" s="6" t="inlineStr">
@@ -4637,6 +5068,11 @@
           <t>Need pincode field mapped in orders and users APIs to track sales, cohorts, and slot trends.</t>
         </is>
       </c>
+      <c r="J88" s="6" t="inlineStr">
+        <is>
+          <t>3. Store Operations &amp; 2. User Analytics</t>
+        </is>
+      </c>
     </row>
     <row r="89" ht="42" customHeight="1">
       <c r="A89" s="3" t="inlineStr">
@@ -4684,6 +5120,11 @@
           <t>Need pincode field mapped in orders and users APIs to track sales, cohorts, and slot trends.</t>
         </is>
       </c>
+      <c r="J89" s="3" t="inlineStr">
+        <is>
+          <t>3. Store Operations &amp; 2. User Analytics</t>
+        </is>
+      </c>
     </row>
     <row r="90" ht="42" customHeight="1">
       <c r="A90" s="6" t="inlineStr">
@@ -4731,6 +5172,11 @@
           <t>Need pincode field mapped in orders and users APIs to track sales, cohorts, and slot trends.</t>
         </is>
       </c>
+      <c r="J90" s="6" t="inlineStr">
+        <is>
+          <t>3. Store Operations &amp; 2. User Analytics</t>
+        </is>
+      </c>
     </row>
     <row r="91" ht="42" customHeight="1">
       <c r="A91" s="3" t="inlineStr">
@@ -4778,6 +5224,11 @@
           <t>Need pincode field mapped in orders and users APIs to track sales, cohorts, and slot trends.</t>
         </is>
       </c>
+      <c r="J91" s="3" t="inlineStr">
+        <is>
+          <t>3. Store Operations &amp; 2. User Analytics</t>
+        </is>
+      </c>
     </row>
     <row r="92" ht="42" customHeight="1">
       <c r="A92" s="6" t="inlineStr">
@@ -4825,6 +5276,11 @@
           <t>None. Handled by existing data schema.</t>
         </is>
       </c>
+      <c r="J92" s="6" t="inlineStr">
+        <is>
+          <t>3. Store Operations, 4. Rider Logistics, 5. Finance &amp; Revenue, 9. Ironer &amp; Staff Performance</t>
+        </is>
+      </c>
     </row>
     <row r="93" ht="42" customHeight="1">
       <c r="A93" s="3" t="inlineStr">
@@ -4872,6 +5328,11 @@
           <t>None. Handled by existing data schema.</t>
         </is>
       </c>
+      <c r="J93" s="3" t="inlineStr">
+        <is>
+          <t>3. Store Operations, 4. Rider Logistics, 5. Finance &amp; Revenue, 9. Ironer &amp; Staff Performance</t>
+        </is>
+      </c>
     </row>
     <row r="94" ht="42" customHeight="1">
       <c r="A94" s="6" t="inlineStr">
@@ -4919,6 +5380,11 @@
           <t>Requires coordinate tracking from rider app and mapping SDK integrations.</t>
         </is>
       </c>
+      <c r="J94" s="6" t="inlineStr">
+        <is>
+          <t>4. Rider Logistics</t>
+        </is>
+      </c>
     </row>
     <row r="95" ht="42" customHeight="1">
       <c r="A95" s="3" t="inlineStr">
@@ -4966,6 +5432,11 @@
           <t>Requires coordinate tracking from rider app and mapping SDK integrations.</t>
         </is>
       </c>
+      <c r="J95" s="3" t="inlineStr">
+        <is>
+          <t>4. Rider Logistics</t>
+        </is>
+      </c>
     </row>
     <row r="96" ht="42" customHeight="1">
       <c r="A96" s="6" t="inlineStr">
@@ -5013,6 +5484,11 @@
           <t>None. Handled by existing data schema.</t>
         </is>
       </c>
+      <c r="J96" s="6" t="inlineStr">
+        <is>
+          <t>3. Store Operations, 4. Rider Logistics, 5. Finance &amp; Revenue, 9. Ironer &amp; Staff Performance</t>
+        </is>
+      </c>
     </row>
     <row r="97" ht="42" customHeight="1">
       <c r="A97" s="3" t="inlineStr">
@@ -5060,6 +5536,11 @@
           <t>None. Handled by existing data schema.</t>
         </is>
       </c>
+      <c r="J97" s="3" t="inlineStr">
+        <is>
+          <t>3. Store Operations, 4. Rider Logistics, 5. Finance &amp; Revenue, 9. Ironer &amp; Staff Performance</t>
+        </is>
+      </c>
     </row>
     <row r="98" ht="42" customHeight="1">
       <c r="A98" s="6" t="inlineStr">
@@ -5107,6 +5588,11 @@
           <t>Reconciliation workflow of rider cash matches needs database structure.</t>
         </is>
       </c>
+      <c r="J98" s="6" t="inlineStr">
+        <is>
+          <t>3. Store Operations, 4. Rider Logistics, 5. Finance &amp; Revenue, 9. Ironer &amp; Staff Performance</t>
+        </is>
+      </c>
     </row>
     <row r="99" ht="42" customHeight="1">
       <c r="A99" s="3" t="inlineStr">
@@ -5154,6 +5640,11 @@
           <t>None. Handled by existing data schema.</t>
         </is>
       </c>
+      <c r="J99" s="3" t="inlineStr">
+        <is>
+          <t>3. Store Operations, 4. Rider Logistics, 5. Finance &amp; Revenue, 9. Ironer &amp; Staff Performance</t>
+        </is>
+      </c>
     </row>
     <row r="100" ht="42" customHeight="1">
       <c r="A100" s="6" t="inlineStr">
@@ -5201,6 +5692,11 @@
           <t>None.</t>
         </is>
       </c>
+      <c r="J100" s="6" t="inlineStr">
+        <is>
+          <t>1. Overview Hub, 2. User Analytics, 3. Store Operations, 7. Complaint &amp; Quality</t>
+        </is>
+      </c>
     </row>
     <row r="101" ht="42" customHeight="1">
       <c r="A101" s="3" t="inlineStr">
@@ -5248,6 +5744,11 @@
           <t>None.</t>
         </is>
       </c>
+      <c r="J101" s="3" t="inlineStr">
+        <is>
+          <t>2. User Analytics, 5. Finance &amp; Revenue, 7. Complaint &amp; Quality</t>
+        </is>
+      </c>
     </row>
     <row r="102" ht="42" customHeight="1">
       <c r="A102" s="6" t="inlineStr">
@@ -5295,6 +5796,11 @@
           <t>None.</t>
         </is>
       </c>
+      <c r="J102" s="6" t="inlineStr">
+        <is>
+          <t>2. User Analytics, 5. Finance &amp; Revenue, 7. Complaint &amp; Quality</t>
+        </is>
+      </c>
     </row>
     <row r="103" ht="42" customHeight="1">
       <c r="A103" s="3" t="inlineStr">
@@ -5342,6 +5848,11 @@
           <t>None.</t>
         </is>
       </c>
+      <c r="J103" s="3" t="inlineStr">
+        <is>
+          <t>2. User Analytics, 5. Finance &amp; Revenue, 7. Complaint &amp; Quality</t>
+        </is>
+      </c>
     </row>
     <row r="104" ht="42" customHeight="1">
       <c r="A104" s="6" t="inlineStr">
@@ -5389,6 +5900,11 @@
           <t>No digital marketing spend tracking exists. Blocked by missing marketing spend table.</t>
         </is>
       </c>
+      <c r="J104" s="6" t="inlineStr">
+        <is>
+          <t>7. Complaint &amp; Quality</t>
+        </is>
+      </c>
     </row>
     <row r="105" ht="42" customHeight="1">
       <c r="A105" s="3" t="inlineStr">
@@ -5436,6 +5952,11 @@
           <t>Needs bag inventory scans inside stores (received list vs delivery-pending bags).</t>
         </is>
       </c>
+      <c r="J105" s="3" t="inlineStr">
+        <is>
+          <t>3. Store Operations</t>
+        </is>
+      </c>
     </row>
     <row r="106" ht="42" customHeight="1">
       <c r="A106" s="6" t="inlineStr">
@@ -5483,6 +6004,11 @@
           <t>Needs bag inventory scans inside stores (received list vs delivery-pending bags).</t>
         </is>
       </c>
+      <c r="J106" s="6" t="inlineStr">
+        <is>
+          <t>3. Store Operations</t>
+        </is>
+      </c>
     </row>
     <row r="107" ht="42" customHeight="1">
       <c r="A107" s="3" t="inlineStr">
@@ -5530,6 +6056,11 @@
           <t>Need backend automated billing and invoice PDF generation.</t>
         </is>
       </c>
+      <c r="J107" s="3" t="inlineStr">
+        <is>
+          <t>5. Finance &amp; Revenue</t>
+        </is>
+      </c>
     </row>
     <row r="108" ht="42" customHeight="1">
       <c r="A108" s="6" t="inlineStr">
@@ -5577,6 +6108,11 @@
           <t>None. Handled by existing data schema.</t>
         </is>
       </c>
+      <c r="J108" s="6" t="inlineStr">
+        <is>
+          <t>1. Overview Hub, 2. User Analytics, 3. Store Operations, 5. Finance &amp; Revenue, 11. Operational Lists &amp; Tables</t>
+        </is>
+      </c>
     </row>
     <row r="109" ht="42" customHeight="1">
       <c r="A109" s="3" t="inlineStr">
@@ -5624,6 +6160,11 @@
           <t>None. Handled by existing data schema.</t>
         </is>
       </c>
+      <c r="J109" s="3" t="inlineStr">
+        <is>
+          <t>1. Overview Hub, 2. User Analytics, 3. Store Operations, 5. Finance &amp; Revenue, 11. Operational Lists &amp; Tables</t>
+        </is>
+      </c>
     </row>
     <row r="110" ht="42" customHeight="1">
       <c r="A110" s="6" t="inlineStr">
@@ -5671,6 +6212,11 @@
           <t>None. Handled by existing data schema.</t>
         </is>
       </c>
+      <c r="J110" s="6" t="inlineStr">
+        <is>
+          <t>1. Overview Hub, 2. User Analytics, 5. Finance &amp; Revenue, 11. Operational Lists &amp; Tables</t>
+        </is>
+      </c>
     </row>
     <row r="111" ht="42" customHeight="1">
       <c r="A111" s="3" t="inlineStr">
@@ -5718,6 +6264,11 @@
           <t>None. Handled by existing data schema.</t>
         </is>
       </c>
+      <c r="J111" s="3" t="inlineStr">
+        <is>
+          <t>1. Overview Hub, 2. User Analytics, 3. Store Operations, 5. Finance &amp; Revenue, 11. Operational Lists &amp; Tables</t>
+        </is>
+      </c>
     </row>
     <row r="112" ht="42" customHeight="1">
       <c r="A112" s="6" t="inlineStr">
@@ -5765,6 +6316,11 @@
           <t>None. Handled by existing data schema.</t>
         </is>
       </c>
+      <c r="J112" s="6" t="inlineStr">
+        <is>
+          <t>1. Overview Hub, 2. User Analytics, 3. Store Operations, 5. Finance &amp; Revenue, 11. Operational Lists &amp; Tables</t>
+        </is>
+      </c>
     </row>
     <row r="113" ht="42" customHeight="1">
       <c r="A113" s="3" t="inlineStr">
@@ -5812,6 +6368,11 @@
           <t>None. Handled by existing data schema.</t>
         </is>
       </c>
+      <c r="J113" s="3" t="inlineStr">
+        <is>
+          <t>1. Overview Hub, 2. User Analytics, 3. Store Operations, 5. Finance &amp; Revenue, 11. Operational Lists &amp; Tables</t>
+        </is>
+      </c>
     </row>
     <row r="114" ht="42" customHeight="1">
       <c r="A114" s="6" t="inlineStr">
@@ -5859,10 +6420,15 @@
           <t>None. Handled by existing data schema.</t>
         </is>
       </c>
+      <c r="J114" s="6" t="inlineStr">
+        <is>
+          <t>1. Overview Hub, 2. User Analytics, 3. Store Operations, 7. Complaint &amp; Quality</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A1:J1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>